<commit_message>
proiectul de baza pentru Poker
</commit_message>
<xml_diff>
--- a/Algoritmi Fundamentali/Prezenta.xlsx
+++ b/Algoritmi Fundamentali/Prezenta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\remus\Documents\GitHub\Facultate_Promotia_2025_2028\Algoritmi Fundamentali\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B0BD606-2AE5-4EF2-B6FF-786607C7A29C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69C852F3-D317-4EF6-98B6-1204C349F77A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>Prenume Nume</t>
   </si>
@@ -124,6 +124,15 @@
   </si>
   <si>
     <t>Beatrix Pont</t>
+  </si>
+  <si>
+    <t>Filip Claudiu Samu</t>
+  </si>
+  <si>
+    <t>Catalin Nae</t>
+  </si>
+  <si>
+    <t>Istvan Gal</t>
   </si>
 </sst>
 </file>
@@ -729,12 +738,14 @@
     </row>
     <row r="3" spans="2:19">
       <c r="B3" s="4" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="C3" s="5">
         <v>1</v>
       </c>
-      <c r="D3" s="6"/>
+      <c r="D3" s="6">
+        <v>1</v>
+      </c>
       <c r="E3" s="6"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
@@ -748,22 +759,22 @@
       <c r="O3" s="6"/>
       <c r="P3" s="7"/>
       <c r="Q3" s="8">
-        <f t="shared" ref="Q3:Q34" si="0">C3+D3+E3+F3+G3+H3+I3+J3+K3+L3+M3+N3+O3+P3</f>
-        <v>1</v>
+        <f>C3+D3+E3+F3+G3+H3+I3+J3+K3+L3+M3+N3+O3+P3</f>
+        <v>2</v>
       </c>
       <c r="R3" s="5"/>
       <c r="S3" s="7"/>
     </row>
     <row r="4" spans="2:19">
       <c r="B4" s="4" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C4" s="9">
         <v>1</v>
       </c>
       <c r="P4" s="10"/>
       <c r="Q4" s="8">
-        <f t="shared" si="0"/>
+        <f>C4+D4+E4+F4+G4+H4+I4+J4+K4+L4+M4+N4+O4+P4</f>
         <v>1</v>
       </c>
       <c r="R4" s="9"/>
@@ -771,29 +782,32 @@
     </row>
     <row r="5" spans="2:19">
       <c r="B5" s="4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C5" s="9">
+        <v>1</v>
+      </c>
+      <c r="D5" s="3">
         <v>1</v>
       </c>
       <c r="P5" s="10"/>
       <c r="Q5" s="8">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f>C5+D5+E5+F5+G5+H5+I5+J5+K5+L5+M5+N5+O5+P5</f>
+        <v>2</v>
       </c>
       <c r="R5" s="9"/>
       <c r="S5" s="10"/>
     </row>
     <row r="6" spans="2:19">
       <c r="B6" s="4" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="C6" s="9">
         <v>1</v>
       </c>
       <c r="P6" s="10"/>
       <c r="Q6" s="8">
-        <f t="shared" si="0"/>
+        <f>C6+D6+E6+F6+G6+H6+I6+J6+K6+L6+M6+N6+O6+P6</f>
         <v>1</v>
       </c>
       <c r="R6" s="9"/>
@@ -801,14 +815,14 @@
     </row>
     <row r="7" spans="2:19">
       <c r="B7" s="4" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="C7" s="9">
         <v>1</v>
       </c>
       <c r="P7" s="10"/>
       <c r="Q7" s="8">
-        <f t="shared" si="0"/>
+        <f>C7+D7+E7+F7+G7+H7+I7+J7+K7+L7+M7+N7+O7+P7</f>
         <v>1</v>
       </c>
       <c r="R7" s="9"/>
@@ -816,14 +830,15 @@
     </row>
     <row r="8" spans="2:19">
       <c r="B8" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C8" s="9">
+        <v>34</v>
+      </c>
+      <c r="C8" s="9"/>
+      <c r="D8" s="3">
         <v>1</v>
       </c>
       <c r="P8" s="10"/>
       <c r="Q8" s="8">
-        <f t="shared" si="0"/>
+        <f>C8+D8+E8+F8+G8+H8+I8+J8+K8+L8+M8+N8+O8+P8</f>
         <v>1</v>
       </c>
       <c r="R8" s="9"/>
@@ -831,29 +846,32 @@
     </row>
     <row r="9" spans="2:19">
       <c r="B9" s="4" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C9" s="9">
+        <v>1</v>
+      </c>
+      <c r="D9" s="3">
         <v>1</v>
       </c>
       <c r="P9" s="10"/>
       <c r="Q9" s="8">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f>C9+D9+E9+F9+G9+H9+I9+J9+K9+L9+M9+N9+O9+P9</f>
+        <v>2</v>
       </c>
       <c r="R9" s="9"/>
       <c r="S9" s="10"/>
     </row>
     <row r="10" spans="2:19">
       <c r="B10" s="4" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C10" s="9">
         <v>1</v>
       </c>
       <c r="P10" s="10"/>
       <c r="Q10" s="8">
-        <f t="shared" si="0"/>
+        <f>C10+D10+E10+F10+G10+H10+I10+J10+K10+L10+M10+N10+O10+P10</f>
         <v>1</v>
       </c>
       <c r="R10" s="9"/>
@@ -861,14 +879,15 @@
     </row>
     <row r="11" spans="2:19">
       <c r="B11" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11" s="9">
+        <v>33</v>
+      </c>
+      <c r="C11" s="9"/>
+      <c r="D11" s="3">
         <v>1</v>
       </c>
       <c r="P11" s="10"/>
       <c r="Q11" s="8">
-        <f t="shared" si="0"/>
+        <f>C11+D11+E11+F11+G11+H11+I11+J11+K11+L11+M11+N11+O11+P11</f>
         <v>1</v>
       </c>
       <c r="R11" s="9"/>
@@ -876,14 +895,14 @@
     </row>
     <row r="12" spans="2:19">
       <c r="B12" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C12" s="9">
         <v>1</v>
       </c>
       <c r="P12" s="10"/>
       <c r="Q12" s="8">
-        <f t="shared" si="0"/>
+        <f>C12+D12+E12+F12+G12+H12+I12+J12+K12+L12+M12+N12+O12+P12</f>
         <v>1</v>
       </c>
       <c r="R12" s="9"/>
@@ -891,29 +910,33 @@
     </row>
     <row r="13" spans="2:19">
       <c r="B13" s="4" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C13" s="9">
+        <v>1</v>
+      </c>
+      <c r="D13" s="3">
         <v>1</v>
       </c>
       <c r="P13" s="10"/>
       <c r="Q13" s="8">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f>C13+D13+E13+F13+G13+H13+I13+J13+K13+L13+M13+N13+O13+P13</f>
+        <v>2</v>
       </c>
       <c r="R13" s="9"/>
       <c r="S13" s="10"/>
     </row>
     <row r="14" spans="2:19">
       <c r="B14" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C14" s="9">
+        <v>35</v>
+      </c>
+      <c r="C14" s="9"/>
+      <c r="D14" s="3">
         <v>1</v>
       </c>
       <c r="P14" s="10"/>
       <c r="Q14" s="8">
-        <f t="shared" si="0"/>
+        <f>C14+D14+E14+F14+G14+H14+I14+J14+K14+L14+M14+N14+O14+P14</f>
         <v>1</v>
       </c>
       <c r="R14" s="9"/>
@@ -921,14 +944,14 @@
     </row>
     <row r="15" spans="2:19">
       <c r="B15" s="4" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="C15" s="9">
         <v>1</v>
       </c>
       <c r="P15" s="10"/>
       <c r="Q15" s="8">
-        <f t="shared" si="0"/>
+        <f>C15+D15+E15+F15+G15+H15+I15+J15+K15+L15+M15+N15+O15+P15</f>
         <v>1</v>
       </c>
       <c r="R15" s="9"/>
@@ -936,63 +959,81 @@
     </row>
     <row r="16" spans="2:19">
       <c r="B16" s="4" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="C16" s="9">
+        <v>1</v>
+      </c>
+      <c r="D16" s="3">
         <v>1</v>
       </c>
       <c r="P16" s="10"/>
       <c r="Q16" s="8">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f>C16+D16+E16+F16+G16+H16+I16+J16+K16+L16+M16+N16+O16+P16</f>
+        <v>2</v>
       </c>
       <c r="R16" s="9"/>
       <c r="S16" s="10"/>
     </row>
     <row r="17" spans="2:19">
       <c r="B17" s="4" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="C17" s="9">
         <v>1</v>
       </c>
       <c r="P17" s="10"/>
       <c r="Q17" s="8">
-        <f t="shared" si="0"/>
+        <f>C17+D17+E17+F17+G17+H17+I17+J17+K17+L17+M17+N17+O17+P17</f>
         <v>1</v>
       </c>
       <c r="R17" s="9"/>
       <c r="S17" s="10"/>
     </row>
     <row r="18" spans="2:19">
-      <c r="B18" s="4"/>
-      <c r="C18" s="9"/>
+      <c r="B18" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" s="9">
+        <v>1</v>
+      </c>
+      <c r="D18" s="3">
+        <v>1</v>
+      </c>
       <c r="P18" s="10"/>
       <c r="Q18" s="8">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>C18+D18+E18+F18+G18+H18+I18+J18+K18+L18+M18+N18+O18+P18</f>
+        <v>2</v>
       </c>
       <c r="R18" s="9"/>
       <c r="S18" s="10"/>
     </row>
     <row r="19" spans="2:19">
-      <c r="B19" s="4"/>
-      <c r="C19" s="9"/>
+      <c r="B19" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" s="9">
+        <v>1</v>
+      </c>
       <c r="P19" s="10"/>
       <c r="Q19" s="8">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>C19+D19+E19+F19+G19+H19+I19+J19+K19+L19+M19+N19+O19+P19</f>
+        <v>1</v>
       </c>
       <c r="R19" s="9"/>
       <c r="S19" s="10"/>
     </row>
     <row r="20" spans="2:19">
-      <c r="B20" s="4"/>
-      <c r="C20" s="9"/>
+      <c r="B20" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20" s="9">
+        <v>1</v>
+      </c>
       <c r="P20" s="10"/>
       <c r="Q20" s="8">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>C20+D20+E20+F20+G20+H20+I20+J20+K20+L20+M20+N20+O20+P20</f>
+        <v>1</v>
       </c>
       <c r="R20" s="9"/>
       <c r="S20" s="10"/>
@@ -1002,7 +1043,7 @@
       <c r="C21" s="9"/>
       <c r="P21" s="10"/>
       <c r="Q21" s="8">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="Q18:Q34" si="0">C21+D21+E21+F21+G21+H21+I21+J21+K21+L21+M21+N21+O21+P21</f>
         <v>0</v>
       </c>
       <c r="R21" s="9"/>
@@ -1417,8 +1458,8 @@
       <c r="S57" s="14"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:S57">
-    <sortCondition ref="B57"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:S20">
+    <sortCondition ref="B20"/>
   </sortState>
   <conditionalFormatting sqref="Q3:Q57">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">

</xml_diff>

<commit_message>
baza proiectului de parcurgere a matricilor
</commit_message>
<xml_diff>
--- a/Algoritmi Fundamentali/Prezenta.xlsx
+++ b/Algoritmi Fundamentali/Prezenta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\remus\Documents\GitHub\Facultate_Promotia_2025_2028\Algoritmi Fundamentali\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{397180AB-D712-4920-9805-926B56BC7E55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECDC1B35-EA59-431F-A52F-E9D85B8C2A59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t>Prenume Nume</t>
   </si>
@@ -154,6 +154,12 @@
   </si>
   <si>
     <t>Radu Răduț</t>
+  </si>
+  <si>
+    <t>Roland Kecskes</t>
+  </si>
+  <si>
+    <t>Robert Barta</t>
   </si>
 </sst>
 </file>
@@ -770,7 +776,9 @@
       <c r="E3" s="6">
         <v>1</v>
       </c>
-      <c r="F3" s="6"/>
+      <c r="F3" s="6">
+        <v>1</v>
+      </c>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
       <c r="I3" s="6"/>
@@ -782,8 +790,8 @@
       <c r="O3" s="6"/>
       <c r="P3" s="7"/>
       <c r="Q3" s="8">
-        <f t="shared" ref="Q3:Q27" si="0">C3+D3+E3+F3+G3+H3+I3+J3+K3+L3+M3+N3+O3+P3</f>
-        <v>3</v>
+        <f>C3+D3+E3+F3+G3+H3+I3+J3+K3+L3+M3+N3+O3+P3</f>
+        <v>4</v>
       </c>
       <c r="R3" s="5"/>
       <c r="S3" s="7"/>
@@ -797,7 +805,7 @@
       </c>
       <c r="P4" s="10"/>
       <c r="Q4" s="8">
-        <f t="shared" si="0"/>
+        <f>C4+D4+E4+F4+G4+H4+I4+J4+K4+L4+M4+N4+O4+P4</f>
         <v>1</v>
       </c>
       <c r="R4" s="9"/>
@@ -818,7 +826,7 @@
       </c>
       <c r="P5" s="10"/>
       <c r="Q5" s="8">
-        <f t="shared" si="0"/>
+        <f>C5+D5+E5+F5+G5+H5+I5+J5+K5+L5+M5+N5+O5+P5</f>
         <v>3</v>
       </c>
       <c r="R5" s="9"/>
@@ -832,10 +840,13 @@
       <c r="E6" s="3">
         <v>1</v>
       </c>
+      <c r="F6" s="3">
+        <v>1</v>
+      </c>
       <c r="P6" s="10"/>
       <c r="Q6" s="8">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f>C6+D6+E6+F6+G6+H6+I6+J6+K6+L6+M6+N6+O6+P6</f>
+        <v>2</v>
       </c>
       <c r="R6" s="9"/>
       <c r="S6" s="10"/>
@@ -855,7 +866,7 @@
       </c>
       <c r="P7" s="10"/>
       <c r="Q7" s="8">
-        <f t="shared" si="0"/>
+        <f>C7+D7+E7+F7+G7+H7+I7+J7+K7+L7+M7+N7+O7+P7</f>
         <v>3</v>
       </c>
       <c r="R7" s="9"/>
@@ -870,7 +881,7 @@
       </c>
       <c r="P8" s="10"/>
       <c r="Q8" s="8">
-        <f t="shared" si="0"/>
+        <f>C8+D8+E8+F8+G8+H8+I8+J8+K8+L8+M8+N8+O8+P8</f>
         <v>1</v>
       </c>
       <c r="R8" s="9"/>
@@ -886,7 +897,7 @@
       </c>
       <c r="P9" s="10"/>
       <c r="Q9" s="8">
-        <f t="shared" si="0"/>
+        <f>C9+D9+E9+F9+G9+H9+I9+J9+K9+L9+M9+N9+O9+P9</f>
         <v>1</v>
       </c>
       <c r="R9" s="9"/>
@@ -905,10 +916,13 @@
       <c r="E10" s="3">
         <v>1</v>
       </c>
+      <c r="F10" s="3">
+        <v>1</v>
+      </c>
       <c r="P10" s="10"/>
       <c r="Q10" s="8">
-        <f t="shared" si="0"/>
-        <v>3</v>
+        <f>C10+D10+E10+F10+G10+H10+I10+J10+K10+L10+M10+N10+O10+P10</f>
+        <v>4</v>
       </c>
       <c r="R10" s="9"/>
       <c r="S10" s="10"/>
@@ -923,7 +937,7 @@
       </c>
       <c r="P11" s="10"/>
       <c r="Q11" s="8">
-        <f t="shared" si="0"/>
+        <f>C11+D11+E11+F11+G11+H11+I11+J11+K11+L11+M11+N11+O11+P11</f>
         <v>1</v>
       </c>
       <c r="R11" s="9"/>
@@ -942,10 +956,13 @@
       <c r="E12" s="3">
         <v>1</v>
       </c>
+      <c r="F12" s="3">
+        <v>1</v>
+      </c>
       <c r="P12" s="10"/>
       <c r="Q12" s="8">
-        <f t="shared" si="0"/>
-        <v>3</v>
+        <f>C12+D12+E12+F12+G12+H12+I12+J12+K12+L12+M12+N12+O12+P12</f>
+        <v>4</v>
       </c>
       <c r="R12" s="9"/>
       <c r="S12" s="10"/>
@@ -958,10 +975,13 @@
       <c r="D13" s="3">
         <v>1</v>
       </c>
+      <c r="F13" s="3">
+        <v>1</v>
+      </c>
       <c r="P13" s="10"/>
       <c r="Q13" s="8">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f>C13+D13+E13+F13+G13+H13+I13+J13+K13+L13+M13+N13+O13+P13</f>
+        <v>2</v>
       </c>
       <c r="R13" s="9"/>
       <c r="S13" s="10"/>
@@ -976,10 +996,13 @@
       <c r="E14" s="3">
         <v>1</v>
       </c>
+      <c r="F14" s="3">
+        <v>1</v>
+      </c>
       <c r="P14" s="10"/>
       <c r="Q14" s="8">
-        <f t="shared" si="0"/>
-        <v>2</v>
+        <f>C14+D14+E14+F14+G14+H14+I14+J14+K14+L14+M14+N14+O14+P14</f>
+        <v>3</v>
       </c>
       <c r="R14" s="9"/>
       <c r="S14" s="10"/>
@@ -997,10 +1020,13 @@
       <c r="E15" s="3">
         <v>1</v>
       </c>
+      <c r="F15" s="3">
+        <v>1</v>
+      </c>
       <c r="P15" s="10"/>
       <c r="Q15" s="8">
-        <f t="shared" si="0"/>
-        <v>3</v>
+        <f>C15+D15+E15+F15+G15+H15+I15+J15+K15+L15+M15+N15+O15+P15</f>
+        <v>4</v>
       </c>
       <c r="R15" s="9"/>
       <c r="S15" s="10"/>
@@ -1015,7 +1041,7 @@
       </c>
       <c r="P16" s="10"/>
       <c r="Q16" s="8">
-        <f t="shared" si="0"/>
+        <f>C16+D16+E16+F16+G16+H16+I16+J16+K16+L16+M16+N16+O16+P16</f>
         <v>1</v>
       </c>
       <c r="R16" s="9"/>
@@ -1034,7 +1060,7 @@
       </c>
       <c r="P17" s="10"/>
       <c r="Q17" s="8">
-        <f t="shared" si="0"/>
+        <f>C17+D17+E17+F17+G17+H17+I17+J17+K17+L17+M17+N17+O17+P17</f>
         <v>2</v>
       </c>
       <c r="R17" s="9"/>
@@ -1051,10 +1077,13 @@
       <c r="E18" s="3">
         <v>1</v>
       </c>
+      <c r="F18" s="3">
+        <v>1</v>
+      </c>
       <c r="P18" s="10"/>
       <c r="Q18" s="8">
-        <f t="shared" si="0"/>
-        <v>2</v>
+        <f>C18+D18+E18+F18+G18+H18+I18+J18+K18+L18+M18+N18+O18+P18</f>
+        <v>3</v>
       </c>
       <c r="R18" s="9"/>
       <c r="S18" s="10"/>
@@ -1069,7 +1098,7 @@
       </c>
       <c r="P19" s="10"/>
       <c r="Q19" s="8">
-        <f t="shared" si="0"/>
+        <f>C19+D19+E19+F19+G19+H19+I19+J19+K19+L19+M19+N19+O19+P19</f>
         <v>1</v>
       </c>
       <c r="R19" s="9"/>
@@ -1082,10 +1111,13 @@
       <c r="C20" s="9">
         <v>1</v>
       </c>
+      <c r="F20" s="3">
+        <v>1</v>
+      </c>
       <c r="P20" s="10"/>
       <c r="Q20" s="8">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f>C20+D20+E20+F20+G20+H20+I20+J20+K20+L20+M20+N20+O20+P20</f>
+        <v>2</v>
       </c>
       <c r="R20" s="9"/>
       <c r="S20" s="10"/>
@@ -1100,7 +1132,7 @@
       </c>
       <c r="P21" s="10"/>
       <c r="Q21" s="8">
-        <f t="shared" si="0"/>
+        <f>C21+D21+E21+F21+G21+H21+I21+J21+K21+L21+M21+N21+O21+P21</f>
         <v>1</v>
       </c>
       <c r="R21" s="9"/>
@@ -1121,7 +1153,7 @@
       </c>
       <c r="P22" s="10"/>
       <c r="Q22" s="8">
-        <f t="shared" si="0"/>
+        <f>C22+D22+E22+F22+G22+H22+I22+J22+K22+L22+M22+N22+O22+P22</f>
         <v>3</v>
       </c>
       <c r="R22" s="9"/>
@@ -1137,7 +1169,7 @@
       </c>
       <c r="P23" s="10"/>
       <c r="Q23" s="8">
-        <f t="shared" si="0"/>
+        <f>C23+D23+E23+F23+G23+H23+I23+J23+K23+L23+M23+N23+O23+P23</f>
         <v>1</v>
       </c>
       <c r="R23" s="9"/>
@@ -1152,7 +1184,7 @@
       </c>
       <c r="P24" s="10"/>
       <c r="Q24" s="8">
-        <f t="shared" si="0"/>
+        <f>C24+D24+E24+F24+G24+H24+I24+J24+K24+L24+M24+N24+O24+P24</f>
         <v>1</v>
       </c>
       <c r="R24" s="9"/>
@@ -1160,76 +1192,92 @@
     </row>
     <row r="25" spans="2:19">
       <c r="B25" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C25" s="9">
-        <v>1</v>
-      </c>
-      <c r="D25" s="3">
+        <v>44</v>
+      </c>
+      <c r="C25" s="9"/>
+      <c r="F25" s="3">
         <v>1</v>
       </c>
       <c r="P25" s="10"/>
       <c r="Q25" s="8">
-        <f t="shared" si="0"/>
-        <v>2</v>
+        <f>C25+D25+E25+F25+G25+H25+I25+J25+K25+L25+M25+N25+O25+P25</f>
+        <v>1</v>
       </c>
       <c r="R25" s="9"/>
       <c r="S25" s="10"/>
     </row>
     <row r="26" spans="2:19">
       <c r="B26" s="4" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C26" s="9">
         <v>1</v>
       </c>
       <c r="D26" s="3">
-        <v>1</v>
-      </c>
-      <c r="E26" s="3">
         <v>1</v>
       </c>
       <c r="P26" s="10"/>
       <c r="Q26" s="8">
-        <f t="shared" si="0"/>
-        <v>3</v>
+        <f>C26+D26+E26+F26+G26+H26+I26+J26+K26+L26+M26+N26+O26+P26</f>
+        <v>2</v>
       </c>
       <c r="R26" s="9"/>
       <c r="S26" s="10"/>
     </row>
     <row r="27" spans="2:19">
       <c r="B27" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C27" s="9">
+        <v>43</v>
+      </c>
+      <c r="C27" s="9"/>
+      <c r="F27" s="3">
         <v>1</v>
       </c>
       <c r="P27" s="10"/>
       <c r="Q27" s="8">
-        <f t="shared" si="0"/>
+        <f>C27+D27+E27+F27+G27+H27+I27+J27+K27+L27+M27+N27+O27+P27</f>
         <v>1</v>
       </c>
       <c r="R27" s="9"/>
       <c r="S27" s="10"/>
     </row>
     <row r="28" spans="2:19">
-      <c r="B28" s="4"/>
-      <c r="C28" s="9"/>
+      <c r="B28" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C28" s="9">
+        <v>1</v>
+      </c>
+      <c r="D28" s="3">
+        <v>1</v>
+      </c>
+      <c r="E28" s="3">
+        <v>1</v>
+      </c>
+      <c r="F28" s="3">
+        <v>1</v>
+      </c>
       <c r="P28" s="10"/>
       <c r="Q28" s="8">
-        <f t="shared" ref="Q28:Q34" si="1">C28+D28+E28+F28+G28+H28+I28+J28+K28+L28+M28+N28+O28+P28</f>
-        <v>0</v>
+        <f>C28+D28+E28+F28+G28+H28+I28+J28+K28+L28+M28+N28+O28+P28</f>
+        <v>4</v>
       </c>
       <c r="R28" s="9"/>
       <c r="S28" s="10"/>
     </row>
     <row r="29" spans="2:19">
-      <c r="B29" s="4"/>
-      <c r="C29" s="9"/>
+      <c r="B29" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C29" s="9">
+        <v>1</v>
+      </c>
+      <c r="F29" s="3">
+        <v>1</v>
+      </c>
       <c r="P29" s="10"/>
       <c r="Q29" s="8">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f>C29+D29+E29+F29+G29+H29+I29+J29+K29+L29+M29+N29+O29+P29</f>
+        <v>2</v>
       </c>
       <c r="R29" s="9"/>
       <c r="S29" s="10"/>
@@ -1239,7 +1287,7 @@
       <c r="C30" s="9"/>
       <c r="P30" s="10"/>
       <c r="Q30" s="8">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="Q28:Q34" si="0">C30+D30+E30+F30+G30+H30+I30+J30+K30+L30+M30+N30+O30+P30</f>
         <v>0</v>
       </c>
       <c r="R30" s="9"/>
@@ -1250,7 +1298,7 @@
       <c r="C31" s="9"/>
       <c r="P31" s="10"/>
       <c r="Q31" s="8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="R31" s="9"/>
@@ -1261,7 +1309,7 @@
       <c r="C32" s="9"/>
       <c r="P32" s="10"/>
       <c r="Q32" s="8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="R32" s="9"/>
@@ -1272,7 +1320,7 @@
       <c r="C33" s="9"/>
       <c r="P33" s="10"/>
       <c r="Q33" s="8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="R33" s="9"/>
@@ -1283,7 +1331,7 @@
       <c r="C34" s="9"/>
       <c r="P34" s="10"/>
       <c r="Q34" s="8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="R34" s="9"/>
@@ -1294,7 +1342,7 @@
       <c r="C35" s="9"/>
       <c r="P35" s="10"/>
       <c r="Q35" s="8">
-        <f t="shared" ref="Q35:Q57" si="2">C35+D35+E35+F35+G35+H35+I35+J35+K35+L35+M35+N35+O35+P35</f>
+        <f t="shared" ref="Q35:Q57" si="1">C35+D35+E35+F35+G35+H35+I35+J35+K35+L35+M35+N35+O35+P35</f>
         <v>0</v>
       </c>
       <c r="R35" s="9"/>
@@ -1305,7 +1353,7 @@
       <c r="C36" s="9"/>
       <c r="P36" s="10"/>
       <c r="Q36" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R36" s="9"/>
@@ -1316,7 +1364,7 @@
       <c r="C37" s="9"/>
       <c r="P37" s="10"/>
       <c r="Q37" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R37" s="9"/>
@@ -1327,7 +1375,7 @@
       <c r="C38" s="9"/>
       <c r="P38" s="10"/>
       <c r="Q38" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R38" s="9"/>
@@ -1338,7 +1386,7 @@
       <c r="C39" s="9"/>
       <c r="P39" s="10"/>
       <c r="Q39" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R39" s="9"/>
@@ -1349,7 +1397,7 @@
       <c r="C40" s="9"/>
       <c r="P40" s="10"/>
       <c r="Q40" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R40" s="9"/>
@@ -1360,7 +1408,7 @@
       <c r="C41" s="9"/>
       <c r="P41" s="10"/>
       <c r="Q41" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R41" s="9"/>
@@ -1371,7 +1419,7 @@
       <c r="C42" s="9"/>
       <c r="P42" s="10"/>
       <c r="Q42" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R42" s="9"/>
@@ -1382,7 +1430,7 @@
       <c r="C43" s="9"/>
       <c r="P43" s="10"/>
       <c r="Q43" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R43" s="9"/>
@@ -1393,7 +1441,7 @@
       <c r="C44" s="9"/>
       <c r="P44" s="10"/>
       <c r="Q44" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R44" s="9"/>
@@ -1404,7 +1452,7 @@
       <c r="C45" s="9"/>
       <c r="P45" s="10"/>
       <c r="Q45" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R45" s="9"/>
@@ -1415,7 +1463,7 @@
       <c r="C46" s="9"/>
       <c r="P46" s="10"/>
       <c r="Q46" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R46" s="9"/>
@@ -1426,7 +1474,7 @@
       <c r="C47" s="9"/>
       <c r="P47" s="10"/>
       <c r="Q47" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R47" s="9"/>
@@ -1437,7 +1485,7 @@
       <c r="C48" s="9"/>
       <c r="P48" s="10"/>
       <c r="Q48" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R48" s="9"/>
@@ -1448,7 +1496,7 @@
       <c r="C49" s="9"/>
       <c r="P49" s="10"/>
       <c r="Q49" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R49" s="9"/>
@@ -1459,7 +1507,7 @@
       <c r="C50" s="9"/>
       <c r="P50" s="10"/>
       <c r="Q50" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R50" s="9"/>
@@ -1470,7 +1518,7 @@
       <c r="C51" s="9"/>
       <c r="P51" s="10"/>
       <c r="Q51" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R51" s="9"/>
@@ -1481,7 +1529,7 @@
       <c r="C52" s="9"/>
       <c r="P52" s="10"/>
       <c r="Q52" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R52" s="9"/>
@@ -1492,7 +1540,7 @@
       <c r="C53" s="9"/>
       <c r="P53" s="10"/>
       <c r="Q53" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R53" s="9"/>
@@ -1503,7 +1551,7 @@
       <c r="C54" s="9"/>
       <c r="P54" s="10"/>
       <c r="Q54" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R54" s="9"/>
@@ -1514,7 +1562,7 @@
       <c r="C55" s="9"/>
       <c r="P55" s="10"/>
       <c r="Q55" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R55" s="9"/>
@@ -1525,7 +1573,7 @@
       <c r="C56" s="9"/>
       <c r="P56" s="10"/>
       <c r="Q56" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R56" s="9"/>
@@ -1548,15 +1596,15 @@
       <c r="O57" s="13"/>
       <c r="P57" s="14"/>
       <c r="Q57" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R57" s="12"/>
       <c r="S57" s="14"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:R27">
-    <sortCondition ref="B3:B27"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:Q29">
+    <sortCondition ref="B3:B29"/>
   </sortState>
   <conditionalFormatting sqref="Q3:Q57">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">

</xml_diff>

<commit_message>
Game of life (automate Fredkin)
</commit_message>
<xml_diff>
--- a/Algoritmi Fundamentali/Prezenta.xlsx
+++ b/Algoritmi Fundamentali/Prezenta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\remus\Documents\GitHub\Facultate_Promotia_2025_2028\Algoritmi Fundamentali\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11B6B0B3-E61A-4C9E-93C0-DA1CFE462F59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05F1DD28-8C2B-4714-911E-9C53F22FF13E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -785,7 +785,9 @@
       <c r="H3" s="6">
         <v>1</v>
       </c>
-      <c r="I3" s="6"/>
+      <c r="I3" s="6">
+        <v>1</v>
+      </c>
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>
       <c r="L3" s="6"/>
@@ -795,7 +797,7 @@
       <c r="P3" s="7"/>
       <c r="Q3" s="8">
         <f t="shared" ref="Q3:Q29" si="0">C3+D3+E3+F3+G3+H3+I3+J3+K3+L3+M3+N3+O3+P3</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R3" s="5"/>
       <c r="S3" s="7"/>
@@ -859,10 +861,13 @@
       <c r="H6" s="3">
         <v>1</v>
       </c>
+      <c r="I6" s="3">
+        <v>1</v>
+      </c>
       <c r="P6" s="10"/>
       <c r="Q6" s="8">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R6" s="9"/>
       <c r="S6" s="10"/>
@@ -883,10 +888,13 @@
       <c r="G7" s="3">
         <v>1</v>
       </c>
+      <c r="I7" s="3">
+        <v>1</v>
+      </c>
       <c r="P7" s="10"/>
       <c r="Q7" s="8">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R7" s="9"/>
       <c r="S7" s="10"/>
@@ -950,10 +958,13 @@
       <c r="H10" s="3">
         <v>1</v>
       </c>
+      <c r="I10" s="3">
+        <v>1</v>
+      </c>
       <c r="P10" s="10"/>
       <c r="Q10" s="8">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R10" s="9"/>
       <c r="S10" s="10"/>
@@ -1002,10 +1013,13 @@
       <c r="H12" s="3">
         <v>1</v>
       </c>
+      <c r="I12" s="3">
+        <v>1</v>
+      </c>
       <c r="P12" s="10"/>
       <c r="Q12" s="8">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R12" s="9"/>
       <c r="S12" s="10"/>
@@ -1084,10 +1098,13 @@
       <c r="H15" s="3">
         <v>1</v>
       </c>
+      <c r="I15" s="3">
+        <v>1</v>
+      </c>
       <c r="P15" s="10"/>
       <c r="Q15" s="8">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R15" s="9"/>
       <c r="S15" s="10"/>
@@ -1156,10 +1173,13 @@
       <c r="H18" s="3">
         <v>1</v>
       </c>
+      <c r="I18" s="3">
+        <v>1</v>
+      </c>
       <c r="P18" s="10"/>
       <c r="Q18" s="8">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R18" s="9"/>
       <c r="S18" s="10"/>
@@ -1205,10 +1225,13 @@
       <c r="H20" s="3">
         <v>1</v>
       </c>
+      <c r="I20" s="3">
+        <v>1</v>
+      </c>
       <c r="P20" s="10"/>
       <c r="Q20" s="8">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R20" s="9"/>
       <c r="S20" s="10"/>
@@ -1273,10 +1296,13 @@
       <c r="H23" s="3">
         <v>1</v>
       </c>
+      <c r="I23" s="3">
+        <v>1</v>
+      </c>
       <c r="P23" s="10"/>
       <c r="Q23" s="8">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R23" s="9"/>
       <c r="S23" s="10"/>
@@ -1350,10 +1376,13 @@
       <c r="H27" s="3">
         <v>1</v>
       </c>
+      <c r="I27" s="3">
+        <v>1</v>
+      </c>
       <c r="P27" s="10"/>
       <c r="Q27" s="8">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R27" s="9"/>
       <c r="S27" s="10"/>
@@ -1380,10 +1409,13 @@
       <c r="H28" s="3">
         <v>1</v>
       </c>
+      <c r="I28" s="3">
+        <v>1</v>
+      </c>
       <c r="P28" s="10"/>
       <c r="Q28" s="8">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R28" s="9"/>
       <c r="S28" s="10"/>

</xml_diff>

<commit_message>
calcularea puterii unui vector
</commit_message>
<xml_diff>
--- a/Algoritmi Fundamentali/Prezenta.xlsx
+++ b/Algoritmi Fundamentali/Prezenta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\remus\Documents\GitHub\Facultate_Promotia_2025_2028\Algoritmi Fundamentali\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C208EC27-76B7-4E32-B06B-8D98149AC014}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F68AC91F-B6A6-4041-B7BF-E1DFB356034C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t>Prenume Nume</t>
   </si>
@@ -163,6 +163,9 @@
   </si>
   <si>
     <t>Luca Prajea</t>
+  </si>
+  <si>
+    <t>Antonio Nichitescu</t>
   </si>
 </sst>
 </file>
@@ -794,15 +797,17 @@
       <c r="J3" s="6">
         <v>1</v>
       </c>
-      <c r="K3" s="6"/>
+      <c r="K3" s="6">
+        <v>1</v>
+      </c>
       <c r="L3" s="6"/>
       <c r="M3" s="6"/>
       <c r="N3" s="6"/>
       <c r="O3" s="6"/>
       <c r="P3" s="7"/>
       <c r="Q3" s="8">
-        <f t="shared" ref="Q3:Q29" si="0">C3+D3+E3+F3+G3+H3+I3+J3+K3+L3+M3+N3+O3+P3</f>
-        <v>8</v>
+        <f t="shared" ref="Q3:Q30" si="0">C3+D3+E3+F3+G3+H3+I3+J3+K3+L3+M3+N3+O3+P3</f>
+        <v>9</v>
       </c>
       <c r="R3" s="5"/>
       <c r="S3" s="7"/>
@@ -939,10 +944,13 @@
       <c r="J9" s="3">
         <v>1</v>
       </c>
+      <c r="K9" s="3">
+        <v>1</v>
+      </c>
       <c r="P9" s="10"/>
       <c r="Q9" s="8">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R9" s="9"/>
       <c r="S9" s="10"/>
@@ -975,10 +983,13 @@
       <c r="J10" s="3">
         <v>1</v>
       </c>
+      <c r="K10" s="3">
+        <v>1</v>
+      </c>
       <c r="P10" s="10"/>
       <c r="Q10" s="8">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R10" s="9"/>
       <c r="S10" s="10"/>
@@ -1000,10 +1011,13 @@
       <c r="J11" s="3">
         <v>1</v>
       </c>
+      <c r="K11" s="3">
+        <v>1</v>
+      </c>
       <c r="P11" s="10"/>
       <c r="Q11" s="8">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R11" s="9"/>
       <c r="S11" s="10"/>
@@ -1036,10 +1050,13 @@
       <c r="J12" s="3">
         <v>1</v>
       </c>
+      <c r="K12" s="3">
+        <v>1</v>
+      </c>
       <c r="P12" s="10"/>
       <c r="Q12" s="8">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R12" s="9"/>
       <c r="S12" s="10"/>
@@ -1094,10 +1111,13 @@
       <c r="J14" s="3">
         <v>1</v>
       </c>
+      <c r="K14" s="3">
+        <v>1</v>
+      </c>
       <c r="P14" s="10"/>
       <c r="Q14" s="8">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R14" s="9"/>
       <c r="S14" s="10"/>
@@ -1130,10 +1150,13 @@
       <c r="J15" s="3">
         <v>1</v>
       </c>
+      <c r="K15" s="3">
+        <v>1</v>
+      </c>
       <c r="P15" s="10"/>
       <c r="Q15" s="8">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R15" s="9"/>
       <c r="S15" s="10"/>
@@ -1211,10 +1234,13 @@
       <c r="J18" s="3">
         <v>1</v>
       </c>
+      <c r="K18" s="3">
+        <v>1</v>
+      </c>
       <c r="P18" s="10"/>
       <c r="Q18" s="8">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R18" s="9"/>
       <c r="S18" s="10"/>
@@ -1266,10 +1292,13 @@
       <c r="I20" s="3">
         <v>1</v>
       </c>
+      <c r="K20" s="3">
+        <v>1</v>
+      </c>
       <c r="P20" s="10"/>
       <c r="Q20" s="8">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R20" s="9"/>
       <c r="S20" s="10"/>
@@ -1288,59 +1317,50 @@
       <c r="J21" s="3">
         <v>1</v>
       </c>
+      <c r="K21" s="3">
+        <v>1</v>
+      </c>
       <c r="P21" s="10"/>
       <c r="Q21" s="8">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R21" s="9"/>
       <c r="S21" s="10"/>
     </row>
     <row r="22" spans="2:19">
       <c r="B22" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C22" s="9">
-        <v>1</v>
-      </c>
-      <c r="D22" s="3">
-        <v>1</v>
-      </c>
-      <c r="E22" s="3">
-        <v>1</v>
-      </c>
-      <c r="G22" s="3">
-        <v>1</v>
-      </c>
-      <c r="H22" s="3">
-        <v>1</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="C22" s="9"/>
       <c r="J22" s="3">
         <v>1</v>
       </c>
       <c r="P22" s="10"/>
       <c r="Q22" s="8">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="R22" s="9"/>
       <c r="S22" s="10"/>
     </row>
     <row r="23" spans="2:19">
       <c r="B23" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C23" s="9"/>
+        <v>21</v>
+      </c>
+      <c r="C23" s="9">
+        <v>1</v>
+      </c>
+      <c r="D23" s="3">
+        <v>1</v>
+      </c>
       <c r="E23" s="3">
         <v>1</v>
       </c>
-      <c r="F23" s="3">
+      <c r="G23" s="3">
         <v>1</v>
       </c>
       <c r="H23" s="3">
-        <v>1</v>
-      </c>
-      <c r="I23" s="3">
         <v>1</v>
       </c>
       <c r="J23" s="3">
@@ -1349,38 +1369,47 @@
       <c r="P23" s="10"/>
       <c r="Q23" s="8">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R23" s="9"/>
       <c r="S23" s="10"/>
     </row>
     <row r="24" spans="2:19">
       <c r="B24" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C24" s="9">
+        <v>42</v>
+      </c>
+      <c r="C24" s="9"/>
+      <c r="E24" s="3">
+        <v>1</v>
+      </c>
+      <c r="F24" s="3">
+        <v>1</v>
+      </c>
+      <c r="H24" s="3">
+        <v>1</v>
+      </c>
+      <c r="I24" s="3">
         <v>1</v>
       </c>
       <c r="J24" s="3">
+        <v>1</v>
+      </c>
+      <c r="K24" s="3">
         <v>1</v>
       </c>
       <c r="P24" s="10"/>
       <c r="Q24" s="8">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="R24" s="9"/>
       <c r="S24" s="10"/>
     </row>
     <row r="25" spans="2:19">
       <c r="B25" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C25" s="9"/>
-      <c r="F25" s="3">
-        <v>1</v>
-      </c>
-      <c r="G25" s="3">
+        <v>19</v>
+      </c>
+      <c r="C25" s="9">
         <v>1</v>
       </c>
       <c r="J25" s="3">
@@ -1389,25 +1418,26 @@
       <c r="P25" s="10"/>
       <c r="Q25" s="8">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R25" s="9"/>
       <c r="S25" s="10"/>
     </row>
     <row r="26" spans="2:19">
       <c r="B26" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C26" s="9">
-        <v>1</v>
-      </c>
-      <c r="D26" s="3">
+        <v>44</v>
+      </c>
+      <c r="C26" s="9"/>
+      <c r="F26" s="3">
         <v>1</v>
       </c>
       <c r="G26" s="3">
         <v>1</v>
       </c>
       <c r="J26" s="3">
+        <v>1</v>
+      </c>
+      <c r="K26" s="3">
         <v>1</v>
       </c>
       <c r="P26" s="10"/>
@@ -1420,22 +1450,21 @@
     </row>
     <row r="27" spans="2:19">
       <c r="B27" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C27" s="9"/>
-      <c r="F27" s="3">
+        <v>20</v>
+      </c>
+      <c r="C27" s="9">
+        <v>1</v>
+      </c>
+      <c r="D27" s="3">
         <v>1</v>
       </c>
       <c r="G27" s="3">
         <v>1</v>
       </c>
-      <c r="H27" s="3">
-        <v>1</v>
-      </c>
-      <c r="I27" s="3">
-        <v>1</v>
-      </c>
       <c r="J27" s="3">
+        <v>1</v>
+      </c>
+      <c r="K27" s="3">
         <v>1</v>
       </c>
       <c r="P27" s="10"/>
@@ -1448,17 +1477,9 @@
     </row>
     <row r="28" spans="2:19">
       <c r="B28" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C28" s="9">
-        <v>1</v>
-      </c>
-      <c r="D28" s="3">
-        <v>1</v>
-      </c>
-      <c r="E28" s="3">
-        <v>1</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="C28" s="9"/>
       <c r="F28" s="3">
         <v>1</v>
       </c>
@@ -1472,23 +1493,32 @@
         <v>1</v>
       </c>
       <c r="J28" s="3">
+        <v>1</v>
+      </c>
+      <c r="K28" s="3">
         <v>1</v>
       </c>
       <c r="P28" s="10"/>
       <c r="Q28" s="8">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="R28" s="9"/>
       <c r="S28" s="10"/>
     </row>
     <row r="29" spans="2:19">
       <c r="B29" s="4" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C29" s="9">
         <v>1</v>
       </c>
+      <c r="D29" s="3">
+        <v>1</v>
+      </c>
+      <c r="E29" s="3">
+        <v>1</v>
+      </c>
       <c r="F29" s="3">
         <v>1</v>
       </c>
@@ -1496,39 +1526,58 @@
         <v>1</v>
       </c>
       <c r="H29" s="3">
+        <v>1</v>
+      </c>
+      <c r="I29" s="3">
+        <v>1</v>
+      </c>
+      <c r="J29" s="3">
         <v>1</v>
       </c>
       <c r="P29" s="10"/>
       <c r="Q29" s="8">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="R29" s="9"/>
       <c r="S29" s="10"/>
     </row>
     <row r="30" spans="2:19">
       <c r="B30" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C30" s="9"/>
-      <c r="J30" s="3">
+        <v>29</v>
+      </c>
+      <c r="C30" s="9">
+        <v>1</v>
+      </c>
+      <c r="F30" s="3">
+        <v>1</v>
+      </c>
+      <c r="G30" s="3">
+        <v>1</v>
+      </c>
+      <c r="H30" s="3">
         <v>1</v>
       </c>
       <c r="P30" s="10"/>
       <c r="Q30" s="8">
-        <f t="shared" ref="Q30:Q34" si="1">C30+D30+E30+F30+G30+H30+I30+J30+K30+L30+M30+N30+O30+P30</f>
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>4</v>
       </c>
       <c r="R30" s="9"/>
       <c r="S30" s="10"/>
     </row>
     <row r="31" spans="2:19">
-      <c r="B31" s="4"/>
+      <c r="B31" s="4" t="s">
+        <v>46</v>
+      </c>
       <c r="C31" s="9"/>
+      <c r="K31" s="3">
+        <v>1</v>
+      </c>
       <c r="P31" s="10"/>
       <c r="Q31" s="8">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" ref="Q31:Q34" si="1">C31+D31+E31+F31+G31+H31+I31+J31+K31+L31+M31+N31+O31+P31</f>
+        <v>1</v>
       </c>
       <c r="R31" s="9"/>
       <c r="S31" s="10"/>
@@ -1832,8 +1881,8 @@
       <c r="S57" s="14"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:Q29">
-    <sortCondition ref="B3:B29"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:Q30">
+    <sortCondition ref="B3:B30"/>
   </sortState>
   <conditionalFormatting sqref="Q3:Q57">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">

</xml_diff>